<commit_message>
Update StickerBinStickersCosts v2.xlsx with new cost data
</commit_message>
<xml_diff>
--- a/stikerts/StickerBinStickersCosts v2.xlsx
+++ b/stikerts/StickerBinStickersCosts v2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\liron\Local Sites\ordermachine\app\public\wp-content\plugins\orderMachine\stikerts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F9674F21-5146-47DD-ACEE-751FDD56EB03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{154890AF-DAC3-4B99-9101-747C1CF17685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tier 1 Equipment Costs" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,6 @@
     <sheet name="Amazon" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="410" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="312">
   <si>
     <t>Recurring Overhead — Subscriptions &amp; Monthly Costs</t>
   </si>
@@ -955,9 +954,6 @@
   </si>
   <si>
     <t>gmail account</t>
-  </si>
-  <si>
-    <t>domain</t>
   </si>
   <si>
     <t>210 x 297mm Rectangle, Avery Blank Labels | Avery</t>
@@ -2191,7 +2187,7 @@
     </row>
     <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43" s="51" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="B43" s="18"/>
       <c r="C43" s="17"/>
@@ -2253,7 +2249,7 @@
       </c>
       <c r="B53" s="24">
         <f>'Bin Stickers 100x140 4pk'!B68</f>
-        <v>29.075999999999997</v>
+        <v>27.155999999999999</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>112</v>
@@ -2265,7 +2261,7 @@
       </c>
       <c r="B54" s="26">
         <f>B52-B53</f>
-        <v>-23.075999999999997</v>
+        <v>-21.155999999999999</v>
       </c>
     </row>
     <row r="56" spans="1:4" x14ac:dyDescent="0.3">
@@ -2283,7 +2279,7 @@
       </c>
       <c r="B57" s="28">
         <f>IFERROR(B56/B54,"N/A")</f>
-        <v>-27.357860981105912</v>
+        <v>-29.840707128001512</v>
       </c>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.3">
@@ -2292,7 +2288,7 @@
       </c>
       <c r="B58" s="28">
         <f>IFERROR(B57*'Bin Stickers 100x140 4pk'!B7,"N/A")</f>
-        <v>-109.43144392442365</v>
+        <v>-119.36282851200605</v>
       </c>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.3">
@@ -2305,12 +2301,12 @@
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A64" s="51" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B65">
         <v>180</v>
@@ -2318,7 +2314,7 @@
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="B66">
         <v>20</v>
@@ -2326,7 +2322,7 @@
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B67">
         <v>8</v>
@@ -2334,7 +2330,7 @@
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B68">
         <v>8</v>
@@ -2342,7 +2338,7 @@
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A69" s="51" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B69">
         <v>14</v>
@@ -2946,8 +2942,8 @@
         <v>193</v>
       </c>
       <c r="B65" s="43">
-        <f>'Recurring Overhead'!B35</f>
-        <v>6.7189999999999994</v>
+        <f>'Recurring Overhead'!B34</f>
+        <v>6.2389999999999999</v>
       </c>
       <c r="C65" s="2" t="s">
         <v>194</v>
@@ -2959,7 +2955,7 @@
       </c>
       <c r="B66" s="41">
         <f>B65*B7</f>
-        <v>26.875999999999998</v>
+        <v>24.956</v>
       </c>
     </row>
     <row r="68" spans="1:3" x14ac:dyDescent="0.3">
@@ -2968,7 +2964,7 @@
       </c>
       <c r="B68" s="40">
         <f>B58+B66</f>
-        <v>29.075999999999997</v>
+        <v>27.155999999999999</v>
       </c>
     </row>
     <row r="69" spans="1:3" x14ac:dyDescent="0.3">
@@ -2977,7 +2973,7 @@
       </c>
       <c r="B69" s="42">
         <f>B68/B7</f>
-        <v>7.2689999999999992</v>
+        <v>6.7889999999999997</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.3">
@@ -2998,7 +2994,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E34"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
@@ -3098,241 +3094,230 @@
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="17" t="s">
-        <v>305</v>
-      </c>
-      <c r="B9" s="18"/>
+        <v>304</v>
+      </c>
+      <c r="B9" s="18">
+        <v>7</v>
+      </c>
       <c r="C9" s="17"/>
       <c r="D9" s="1"/>
       <c r="E9">
-        <v>30</v>
+        <f>B9*12</f>
+        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="17" t="s">
-        <v>304</v>
+        <v>15</v>
       </c>
       <c r="B10" s="18">
-        <v>11.8</v>
-      </c>
-      <c r="C10" s="17"/>
-      <c r="D10" s="1"/>
-      <c r="E10">
-        <f>B10*12</f>
-        <v>141.60000000000002</v>
+        <v>0</v>
+      </c>
+      <c r="C10" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>16</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="17" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="18">
-        <v>0</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>16</v>
+        <v>306</v>
+      </c>
+      <c r="B11" s="18"/>
+      <c r="C11" s="17"/>
+      <c r="D11" s="1"/>
+      <c r="E11">
+        <v>250</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="17" t="s">
-        <v>307</v>
-      </c>
-      <c r="B12" s="18"/>
-      <c r="C12" s="17"/>
-      <c r="D12" s="1"/>
+      <c r="A12" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="20">
+        <f>SUM(B6:B10)</f>
+        <v>62.39</v>
+      </c>
       <c r="E12">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="19" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="20">
-        <f>SUM(B6:B11)</f>
-        <v>67.19</v>
-      </c>
-      <c r="E13">
-        <f>SUM(E6:E12)</f>
-        <v>948.34</v>
+        <f>SUM(E6:E11)</f>
+        <v>860.74</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="12" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="68" t="s">
+      <c r="A15" s="68" t="s">
         <v>19</v>
       </c>
-      <c r="B16" s="69"/>
-      <c r="C16" s="69"/>
-      <c r="D16" s="69"/>
+      <c r="B15" s="69"/>
+      <c r="C15" s="69"/>
+      <c r="D15" s="69"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B17" s="16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>22</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B18" s="16" t="s">
-        <v>21</v>
-      </c>
-      <c r="C18" s="16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="16" t="s">
-        <v>23</v>
+      <c r="A18" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B18" s="44">
+        <v>10</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="17" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B19" s="44">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="C19" s="17" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="B20" s="44">
-        <v>40</v>
+        <v>30</v>
+      </c>
+      <c r="B20" s="45">
+        <f>B22</f>
+        <v>1</v>
       </c>
       <c r="C20" s="17" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B21" s="45">
-        <f>B23</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="B22" s="46">
         <v>1</v>
       </c>
-      <c r="C21" s="17" t="s">
-        <v>31</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>32</v>
+      <c r="D22" s="1" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="17" t="s">
-        <v>33</v>
-      </c>
-      <c r="B23" s="46">
-        <v>1</v>
+        <v>35</v>
+      </c>
+      <c r="B23" s="45">
+        <f>IFERROR(B22*4.33/(45/60)*20,0)</f>
+        <v>115.46666666666667</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="B24" s="45">
-        <f>IFERROR(B23*4.33/(45/60)*20,0)</f>
-        <v>115.46666666666667</v>
-      </c>
-      <c r="D24" s="1" t="s">
         <v>36</v>
       </c>
     </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="12" t="s">
+        <v>37</v>
+      </c>
+    </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
-        <v>37</v>
+      <c r="A26" s="16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" s="16" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A27" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="B27" s="16" t="s">
-        <v>38</v>
+      <c r="A27" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B27" s="27">
+        <f>IFERROR($B$12/B18,0)</f>
+        <v>6.2389999999999999</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="17" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B28" s="27">
-        <f>IFERROR($B$13/B19,0)</f>
-        <v>6.7189999999999994</v>
+        <f>IFERROR($B$12/B19,0)</f>
+        <v>1.55975</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="17" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B29" s="27">
-        <f>IFERROR($B$13/B20,0)</f>
-        <v>1.6797499999999999</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B30" s="27">
-        <f>IFERROR($B$13/B21,0)</f>
-        <v>67.19</v>
+        <f>IFERROR($B$12/B20,0)</f>
+        <v>62.39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="47" t="s">
+        <v>24</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="B33" s="47" t="s">
-        <v>24</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A34" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="B34" s="45">
-        <f>INDEX(B19:B21,MATCH(B33,A19:A21,0))</f>
+      <c r="B33" s="45">
+        <f>INDEX(B18:B20,MATCH(B32,A18:A20,0))</f>
         <v>10</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="19" t="s">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="B35" s="20">
-        <f>IFERROR($B$13/B34,0)</f>
-        <v>6.7189999999999994</v>
+      <c r="B34" s="20">
+        <f>IFERROR($B$12/B33,0)</f>
+        <v>6.2389999999999999</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A15:D15"/>
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" sqref="B33" xr:uid="{00000000-0002-0000-0200-000000000000}">
+    <dataValidation type="list" sqref="B32" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"Conservative,Base / Target,Optimistic / Capacity ceiling"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>